<commit_message>
docs: 回填对标表Lululun列 + Lululun博主/人群分析 + Quality1st选题库
</commit_message>
<xml_diff>
--- a/docs/工作/10-市场与竞品/Lululun小红书笔记分析.xlsx
+++ b/docs/工作/10-市场与竞品/Lululun小红书笔记分析.xlsx
@@ -13,6 +13,7 @@
     <sheet name="④长尾意图词" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="⑤全量分类明细" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="⑥维度对比数据" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="⑦博主类型&amp;人群" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -58,6 +59,12 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="14"/>
     </font>
   </fonts>
   <fills count="5">
@@ -109,7 +116,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -132,6 +139,14 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -4939,9 +4954,7 @@
           <t>F·其他/泛护肤</t>
         </is>
       </c>
-      <c r="B38" s="7" t="n">
-        <v/>
-      </c>
+      <c r="B38" s="7" t="n"/>
       <c r="C38" s="7" t="n">
         <v>205</v>
       </c>
@@ -6656,9 +6669,7 @@
           <t>F·其他/泛护肤</t>
         </is>
       </c>
-      <c r="B71" s="8" t="n">
-        <v/>
-      </c>
+      <c r="B71" s="8" t="n"/>
       <c r="C71" s="8" t="n">
         <v>8</v>
       </c>
@@ -6966,9 +6977,7 @@
           <t>F·其他/泛护肤</t>
         </is>
       </c>
-      <c r="B77" s="8" t="n">
-        <v/>
-      </c>
+      <c r="B77" s="8" t="n"/>
       <c r="C77" s="8" t="n">
         <v>4</v>
       </c>
@@ -7015,9 +7024,7 @@
           <t>F·其他/泛护肤</t>
         </is>
       </c>
-      <c r="B78" s="7" t="n">
-        <v/>
-      </c>
+      <c r="B78" s="7" t="n"/>
       <c r="C78" s="7" t="n">
         <v>4</v>
       </c>
@@ -7937,4 +7944,502 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>博主类型 &amp; 客户人群分布</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>一、博主类型分布(按声量占比降序)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>博主类型</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>篇数</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>篇数占比%</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>均互动</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>中位互动</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>声量占比%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>美妆护肤垂类</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>18</v>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>20.7</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>636</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>39</v>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>47.9</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>在日/代购·资讯类</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="n">
+        <v>24</v>
+      </c>
+      <c r="C6" s="8" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>208</v>
+      </c>
+      <c r="E6" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="F6" s="8" t="n">
+        <v>20.9</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>好物/购物分享类</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>23</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>225</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>44</v>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>18.8</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>泛生活/素人KOC</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="n">
+        <v>21</v>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>8.6</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>专业/成分党(医生·老师)</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>220</v>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>229</v>
+      </c>
+      <c r="F9" s="7" t="n">
+        <v>3.7</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>注：类型由昵称+内容+IP信号推断，非平台官方标签，供趋势参考。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>二、客户人群信号(内容提及次数)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>年龄/身份</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="n"/>
+      <c r="C13" s="12" t="n"/>
+      <c r="D13" s="12" t="n"/>
+      <c r="E13" s="12" t="n"/>
+      <c r="F13" s="12" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>熟龄/40+/45(抗老)</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="n">
+        <v>16</v>
+      </c>
+      <c r="D14" s="12" t="n"/>
+      <c r="E14" s="12" t="n"/>
+      <c r="F14" s="12" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>25/25+(抗初老)</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="D15" s="12" t="n"/>
+      <c r="E15" s="12" t="n"/>
+      <c r="F15" s="12" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>学生党</t>
+        </is>
+      </c>
+      <c r="B16" s="13" t="n">
+        <v>8</v>
+      </c>
+      <c r="D16" s="12" t="n"/>
+      <c r="E16" s="12" t="n"/>
+      <c r="F16" s="12" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>宝子/姐妹(泛年轻女性)</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="n">
+        <v>13</v>
+      </c>
+      <c r="D17" s="12" t="n"/>
+      <c r="E17" s="12" t="n"/>
+      <c r="F17" s="12" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>肤质</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="n"/>
+      <c r="C18" s="12" t="n"/>
+      <c r="D18" s="12" t="n"/>
+      <c r="E18" s="12" t="n"/>
+      <c r="F18" s="12" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>干皮</t>
+        </is>
+      </c>
+      <c r="B19" s="13" t="n">
+        <v>13</v>
+      </c>
+      <c r="D19" s="12" t="n"/>
+      <c r="E19" s="12" t="n"/>
+      <c r="F19" s="12" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>油皮/混油</t>
+        </is>
+      </c>
+      <c r="B20" s="13" t="n">
+        <v>16</v>
+      </c>
+      <c r="D20" s="12" t="n"/>
+      <c r="E20" s="12" t="n"/>
+      <c r="F20" s="12" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>敏感肌</t>
+        </is>
+      </c>
+      <c r="B21" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="D21" s="12" t="n"/>
+      <c r="E21" s="12" t="n"/>
+      <c r="F21" s="12" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>痘肌/痘印</t>
+        </is>
+      </c>
+      <c r="B22" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="D22" s="12" t="n"/>
+      <c r="E22" s="12" t="n"/>
+      <c r="F22" s="12" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>使用场景</t>
+        </is>
+      </c>
+      <c r="B23" s="12" t="n"/>
+      <c r="C23" s="12" t="n"/>
+      <c r="D23" s="12" t="n"/>
+      <c r="E23" s="12" t="n"/>
+      <c r="F23" s="12" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>妆前(上妆前打底)</t>
+        </is>
+      </c>
+      <c r="B24" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="D24" s="12" t="n"/>
+      <c r="E24" s="12" t="n"/>
+      <c r="F24" s="12" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>熬夜/急救</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="n">
+        <v>24</v>
+      </c>
+      <c r="D25" s="12" t="n"/>
+      <c r="E25" s="12" t="n"/>
+      <c r="F25" s="12" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>旅行/伴手礼(赴日代购)</t>
+        </is>
+      </c>
+      <c r="B26" s="13" t="n">
+        <v>16</v>
+      </c>
+      <c r="D26" s="12" t="n"/>
+      <c r="E26" s="12" t="n"/>
+      <c r="F26" s="12" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>空调房/换季</t>
+        </is>
+      </c>
+      <c r="B27" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="D27" s="12" t="n"/>
+      <c r="E27" s="12" t="n"/>
+      <c r="F27" s="12" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>性别</t>
+        </is>
+      </c>
+      <c r="B28" s="12" t="n"/>
+      <c r="C28" s="12" t="n"/>
+      <c r="D28" s="12" t="n"/>
+      <c r="E28" s="12" t="n"/>
+      <c r="F28" s="12" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>女性(姐妹/女生/小姐姐)</t>
+        </is>
+      </c>
+      <c r="B29" s="13" t="n">
+        <v>18</v>
+      </c>
+      <c r="D29" s="12" t="n"/>
+      <c r="E29" s="12" t="n"/>
+      <c r="F29" s="12" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>男性(男生/男士)</t>
+        </is>
+      </c>
+      <c r="B30" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="D30" s="12" t="n"/>
+      <c r="E30" s="12" t="n"/>
+      <c r="F30" s="12" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>价格心智</t>
+        </is>
+      </c>
+      <c r="B31" s="12" t="n"/>
+      <c r="C31" s="12" t="n"/>
+      <c r="D31" s="12" t="n"/>
+      <c r="E31" s="12" t="n"/>
+      <c r="F31" s="12" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>平价/便宜</t>
+        </is>
+      </c>
+      <c r="B32" s="13" t="n">
+        <v>43</v>
+      </c>
+      <c r="D32" s="12" t="n"/>
+      <c r="E32" s="12" t="n"/>
+      <c r="F32" s="12" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>性价比</t>
+        </is>
+      </c>
+      <c r="B33" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="D33" s="12" t="n"/>
+      <c r="E33" s="12" t="n"/>
+      <c r="F33" s="12" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>学生党/省钱</t>
+        </is>
+      </c>
+      <c r="B34" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="D34" s="12" t="n"/>
+      <c r="E34" s="12" t="n"/>
+      <c r="F34" s="12" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="23">
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="A28:F28"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B26:C26"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>